<commit_message>
Complete T00 three-seed baseline and final report
</commit_message>
<xml_diff>
--- a/submissions/2A202602759_NguyenMinhHien/results.xlsx
+++ b/submissions/2A202602759_NguyenMinhHien/results.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R0c37271cdcbc4c63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backbones" sheetId="2" r:id="Ra88045a28d824a37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Training" sheetId="3" r:id="R80d3556a756443c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inference" sheetId="4" r:id="R857b4302b34e4697"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Final" sheetId="5" r:id="R7de9271fb17e4409"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PerClass" sheetId="6" r:id="R822b739ebc444f38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Latency" sheetId="7" r:id="R05c66301e2294078"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rcf9a99c06d92431a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backbones" sheetId="2" r:id="Ra86f3ae644b74743"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Training" sheetId="3" r:id="R60e20afee475426c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inference" sheetId="4" r:id="R87cb9afa1a9b4ce0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Final" sheetId="5" r:id="Rb0c561b91cb04389"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PerClass" sheetId="6" r:id="R90ca3b377d6f4fd7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Latency" sheetId="7" r:id="Rd5c951c7626f4153"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -366,51 +366,51 @@
         <x:v>ConvNeXt Tiny + T00 + I00</x:v>
       </x:c>
       <x:c r="D3" s="6" t="n">
-        <x:v>0.9656166767749601</x:v>
+        <x:v>0.9671925183622053</x:v>
       </x:c>
       <x:c r="E3" s="6" t="n">
-        <x:v>0.9675699985689636</x:v>
+        <x:v>0.9687787332408145</x:v>
       </x:c>
       <x:c r="F3" s="6" t="n">
-        <x:v>0.974764756201882</x:v>
+        <x:v>0.975762760193898</x:v>
       </x:c>
       <x:c r="G3" s="6" t="n">
-        <x:v>52.415742768749894</x:v>
+        <x:v>51.73038190256659</x:v>
       </x:c>
       <x:c r="H3" s="6" t="n">
         <x:v>7.047970549865567</x:v>
       </x:c>
       <x:c r="I3" s="6" t="str">
-        <x:v>macro-F1 test std 0.0005; 2 seed; thiếu seed2, chưa chấm I2</x:v>
+        <x:v>macro-F1 test std 0.0021; 3 seed</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="24" customHeight="1">
       <x:c r="A4" s="6" t="str">
-        <x:v>F01 − T00 (sơ bộ)</x:v>
+        <x:v>F01 − T00</x:v>
       </x:c>
       <x:c r="B4" s="6" t="str">
         <x:v>Chênh lệch</x:v>
       </x:c>
       <x:c r="C4" s="6" t="str">
-        <x:v>F01: 3 seed; T00: 2 seed</x:v>
+        <x:v>Mean của 3 seed</x:v>
       </x:c>
       <x:c r="D4" s="6" t="n">
-        <x:v>0.004453169598276907</x:v>
+        <x:v>0.002877328011031688</x:v>
       </x:c>
       <x:c r="E4" s="6" t="n">
-        <x:v>0.00484634178728971</x:v>
+        <x:v>0.0036376071154388123</x:v>
       </x:c>
       <x:c r="F4" s="6" t="n">
-        <x:v>0.0030890599752875225</x:v>
+        <x:v>0.002091055983271528</x:v>
       </x:c>
       <x:c r="G4" s="6" t="n">
-        <x:v>47.03929581138348</x:v>
+        <x:v>47.724656677566784</x:v>
       </x:c>
       <x:c r="H4" s="6" t="n">
         <x:v>1.6629909498988118</x:v>
       </x:c>
       <x:c r="I4" s="6" t="str">
-        <x:v>Chưa đủ 3 seed mốc; không dùng chấm I2</x:v>
+        <x:v>Dương là F01 cao hơn mốc</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="24" customHeight="1">
@@ -2666,33 +2666,58 @@
       <x:c r="B8" s="6" t="str">
         <x:v>ConvNeXt Tiny + T00 + I00</x:v>
       </x:c>
-      <x:c r="C8" s="7" t="str">
+      <x:c r="C8" s="7" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D8" s="6" t="n">
+        <x:v>0.9703442015366956</x:v>
+      </x:c>
+      <x:c r="E8" s="6" t="n">
+        <x:v>0.9711962025845161</x:v>
+      </x:c>
+      <x:c r="F8" s="6" t="n">
+        <x:v>0.9777587681779298</x:v>
+      </x:c>
+      <x:c r="G8" s="6" t="n">
+        <x:v>0.009053852603364653</x:v>
+      </x:c>
+      <x:c r="H8" s="6"/>
+      <x:c r="I8" s="6"/>
+      <x:c r="J8" s="6" t="str">
+        <x:v>Đo trên test fold 0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="24" customHeight="1">
+      <x:c r="A9" s="6" t="str">
+        <x:v>T00</x:v>
+      </x:c>
+      <x:c r="B9" s="6" t="str">
+        <x:v>ConvNeXt Tiny + T00 + I00</x:v>
+      </x:c>
+      <x:c r="C9" s="7" t="str">
         <x:v>mean ± std</x:v>
       </x:c>
-      <x:c r="D8" s="6" t="n">
-        <x:v>0.9656166767749601</x:v>
-      </x:c>
-      <x:c r="E8" s="6" t="n">
-        <x:v>0.9675699985689636</x:v>
-      </x:c>
-      <x:c r="F8" s="6" t="n">
-        <x:v>0.974764756201882</x:v>
-      </x:c>
-      <x:c r="G8" s="6" t="n">
-        <x:v>0.010693666144853108</x:v>
-      </x:c>
-      <x:c r="H8" s="6" t="n">
-        <x:v>0.9675699985689636</x:v>
-      </x:c>
-      <x:c r="I8" s="6" t="n">
-        <x:v>0.000540622250085547</x:v>
-      </x:c>
-      <x:c r="J8" s="6" t="str">
-        <x:v>2 seed; std mẫu (ddof=1); thiếu seed2, chưa chấm I2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="C9" s="8"/>
+      <x:c r="D9" s="6" t="n">
+        <x:v>0.9671925183622053</x:v>
+      </x:c>
+      <x:c r="E9" s="6" t="n">
+        <x:v>0.9687787332408145</x:v>
+      </x:c>
+      <x:c r="F9" s="6" t="n">
+        <x:v>0.975762760193898</x:v>
+      </x:c>
+      <x:c r="G9" s="6" t="n">
+        <x:v>0.010147061631023623</x:v>
+      </x:c>
+      <x:c r="H9" s="6" t="n">
+        <x:v>0.9687787332408145</x:v>
+      </x:c>
+      <x:c r="I9" s="6" t="n">
+        <x:v>0.0021282045788520265</x:v>
+      </x:c>
+      <x:c r="J9" s="6" t="str">
+        <x:v>3 seed; std mẫu (ddof=1)</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="C10" s="8"/>
@@ -4264,16 +4289,16 @@
         <x:v>226</x:v>
       </x:c>
       <x:c r="D56" s="6" t="n">
-        <x:v>0.9552095072226205</x:v>
+        <x:v>0.9728506787330317</x:v>
       </x:c>
       <x:c r="E56" s="6" t="n">
-        <x:v>0.9336283185840708</x:v>
+        <x:v>0.9513274336283186</x:v>
       </x:c>
       <x:c r="F56" s="6" t="n">
-        <x:v>0.9441215779910197</x:v>
+        <x:v>0.9619686800894854</x:v>
       </x:c>
       <x:c r="G56" s="6" t="str">
-        <x:v>mean 2 seed</x:v>
+        <x:v>seed 2</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="24" customHeight="1">
@@ -4287,16 +4312,16 @@
         <x:v>213</x:v>
       </x:c>
       <x:c r="D57" s="6" t="n">
-        <x:v>0.9522820719436351</x:v>
+        <x:v>0.9765258215962441</x:v>
       </x:c>
       <x:c r="E57" s="6" t="n">
-        <x:v>0.9835680751173709</x:v>
+        <x:v>0.9765258215962441</x:v>
       </x:c>
       <x:c r="F57" s="6" t="n">
-        <x:v>0.9676672640382318</x:v>
+        <x:v>0.9765258215962441</x:v>
       </x:c>
       <x:c r="G57" s="6" t="str">
-        <x:v>mean 2 seed</x:v>
+        <x:v>seed 2</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="24" customHeight="1">
@@ -4310,16 +4335,16 @@
         <x:v>207</x:v>
       </x:c>
       <x:c r="D58" s="6" t="n">
-        <x:v>0.98062942638713</x:v>
+        <x:v>0.9802955665024631</x:v>
       </x:c>
       <x:c r="E58" s="6" t="n">
-        <x:v>0.9782608695652174</x:v>
+        <x:v>0.961352657004831</x:v>
       </x:c>
       <x:c r="F58" s="6" t="n">
-        <x:v>0.979442280473968</x:v>
+        <x:v>0.9707317073170733</x:v>
       </x:c>
       <x:c r="G58" s="6" t="str">
-        <x:v>mean 2 seed</x:v>
+        <x:v>seed 2</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="24" customHeight="1">
@@ -4333,16 +4358,16 @@
         <x:v>205</x:v>
       </x:c>
       <x:c r="D59" s="6" t="n">
-        <x:v>0.9901108374384237</x:v>
+        <x:v>0.9950248756218906</x:v>
       </x:c>
       <x:c r="E59" s="6" t="n">
-        <x:v>0.973170731707317</x:v>
+        <x:v>0.975609756097561</x:v>
       </x:c>
       <x:c r="F59" s="6" t="n">
-        <x:v>0.9815541031227305</x:v>
+        <x:v>0.9852216748768473</x:v>
       </x:c>
       <x:c r="G59" s="6" t="str">
-        <x:v>mean 2 seed</x:v>
+        <x:v>seed 2</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="24" customHeight="1">
@@ -4356,16 +4381,16 @@
         <x:v>213</x:v>
       </x:c>
       <x:c r="D60" s="6" t="n">
-        <x:v>0.9283257918552037</x:v>
+        <x:v>0.9196428571428571</x:v>
       </x:c>
       <x:c r="E60" s="6" t="n">
-        <x:v>0.971830985915493</x:v>
+        <x:v>0.9671361502347418</x:v>
       </x:c>
       <x:c r="F60" s="6" t="n">
-        <x:v>0.9495612650716496</x:v>
+        <x:v>0.9427917620137299</x:v>
       </x:c>
       <x:c r="G60" s="6" t="str">
-        <x:v>mean 2 seed</x:v>
+        <x:v>seed 2</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="24" customHeight="1">
@@ -4379,16 +4404,16 @@
         <x:v>202</x:v>
       </x:c>
       <x:c r="D61" s="6" t="n">
-        <x:v>0.9829243303898132</x:v>
+        <x:v>0.9800995024875622</x:v>
       </x:c>
       <x:c r="E61" s="6" t="n">
-        <x:v>0.9851485148514851</x:v>
+        <x:v>0.9752475247524752</x:v>
       </x:c>
       <x:c r="F61" s="6" t="n">
-        <x:v>0.9839616644662852</x:v>
+        <x:v>0.977667493796526</x:v>
       </x:c>
       <x:c r="G61" s="6" t="str">
-        <x:v>mean 2 seed</x:v>
+        <x:v>seed 2</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="24" customHeight="1">
@@ -4402,16 +4427,16 @@
         <x:v>215</x:v>
       </x:c>
       <x:c r="D62" s="6" t="n">
-        <x:v>0.9575375375375376</x:v>
+        <x:v>0.9770642201834863</x:v>
       </x:c>
       <x:c r="E62" s="6" t="n">
-        <x:v>0.9953488372093023</x:v>
+        <x:v>0.9906976744186047</x:v>
       </x:c>
       <x:c r="F62" s="6" t="n">
-        <x:v>0.9760661535261078</x:v>
+        <x:v>0.9838337182448038</x:v>
       </x:c>
       <x:c r="G62" s="6" t="str">
-        <x:v>mean 2 seed</x:v>
+        <x:v>seed 2</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="24" customHeight="1">
@@ -4425,16 +4450,16 @@
         <x:v>204</x:v>
       </x:c>
       <x:c r="D63" s="6" t="n">
-        <x:v>0.9457481582670635</x:v>
+        <x:v>0.9471153846153846</x:v>
       </x:c>
       <x:c r="E63" s="6" t="n">
-        <x:v>0.9387254901960784</x:v>
+        <x:v>0.9656862745098039</x:v>
       </x:c>
       <x:c r="F63" s="6" t="n">
-        <x:v>0.9421533619802699</x:v>
+        <x:v>0.9563106796116505</x:v>
       </x:c>
       <x:c r="G63" s="6" t="str">
-        <x:v>mean 2 seed</x:v>
+        <x:v>seed 2</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="24" customHeight="1">
@@ -4448,44 +4473,224 @@
         <x:v>1822</x:v>
       </x:c>
       <x:c r="D64" s="6" t="n">
-        <x:v>0.987823263578633</x:v>
+        <x:v>0.9867986798679867</x:v>
       </x:c>
       <x:c r="E64" s="6" t="n">
-        <x:v>0.9794182217343579</x:v>
+        <x:v>0.9846322722283205</x:v>
       </x:c>
       <x:c r="F64" s="6" t="n">
-        <x:v>0.9836023164504102</x:v>
+        <x:v>0.9857142857142857</x:v>
       </x:c>
       <x:c r="G64" s="6" t="str">
-        <x:v>mean 2 seed</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="65">
-      <x:c r="C65" s="10"/>
-    </x:row>
-    <x:row r="66">
-      <x:c r="C66" s="10"/>
-    </x:row>
-    <x:row r="67">
-      <x:c r="C67" s="10"/>
-    </x:row>
-    <x:row r="68">
-      <x:c r="C68" s="10"/>
-    </x:row>
-    <x:row r="69">
-      <x:c r="C69" s="10"/>
-    </x:row>
-    <x:row r="70">
-      <x:c r="C70" s="10"/>
-    </x:row>
-    <x:row r="71">
-      <x:c r="C71" s="10"/>
-    </x:row>
-    <x:row r="72">
-      <x:c r="C72" s="10"/>
-    </x:row>
-    <x:row r="73">
-      <x:c r="C73" s="10"/>
+        <x:v>seed 2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="24" customHeight="1">
+      <x:c r="A65" s="6" t="str">
+        <x:v>T00</x:v>
+      </x:c>
+      <x:c r="B65" s="6" t="str">
+        <x:v>Chinee apple</x:v>
+      </x:c>
+      <x:c r="C65" s="9" t="n">
+        <x:v>226</x:v>
+      </x:c>
+      <x:c r="D65" s="6" t="n">
+        <x:v>0.961089897726091</x:v>
+      </x:c>
+      <x:c r="E65" s="6" t="n">
+        <x:v>0.93952802359882</x:v>
+      </x:c>
+      <x:c r="F65" s="6" t="n">
+        <x:v>0.9500706120238416</x:v>
+      </x:c>
+      <x:c r="G65" s="6" t="str">
+        <x:v>mean 3 seed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="24" customHeight="1">
+      <x:c r="A66" s="6" t="str">
+        <x:v>T00</x:v>
+      </x:c>
+      <x:c r="B66" s="6" t="str">
+        <x:v>Lantana</x:v>
+      </x:c>
+      <x:c r="C66" s="9" t="n">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="D66" s="6" t="n">
+        <x:v>0.9603633218278381</x:v>
+      </x:c>
+      <x:c r="E66" s="6" t="n">
+        <x:v>0.9812206572769954</x:v>
+      </x:c>
+      <x:c r="F66" s="6" t="n">
+        <x:v>0.9706201165575692</x:v>
+      </x:c>
+      <x:c r="G66" s="6" t="str">
+        <x:v>mean 3 seed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="24" customHeight="1">
+      <x:c r="A67" s="6" t="str">
+        <x:v>T00</x:v>
+      </x:c>
+      <x:c r="B67" s="6" t="str">
+        <x:v>Parkinsonia</x:v>
+      </x:c>
+      <x:c r="C67" s="9" t="n">
+        <x:v>207</x:v>
+      </x:c>
+      <x:c r="D67" s="6" t="n">
+        <x:v>0.9805181397589077</x:v>
+      </x:c>
+      <x:c r="E67" s="6" t="n">
+        <x:v>0.9726247987117552</x:v>
+      </x:c>
+      <x:c r="F67" s="6" t="n">
+        <x:v>0.9765387560883364</x:v>
+      </x:c>
+      <x:c r="G67" s="6" t="str">
+        <x:v>mean 3 seed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="24" customHeight="1">
+      <x:c r="A68" s="6" t="str">
+        <x:v>T00</x:v>
+      </x:c>
+      <x:c r="B68" s="6" t="str">
+        <x:v>Parthenium</x:v>
+      </x:c>
+      <x:c r="C68" s="9" t="n">
+        <x:v>205</x:v>
+      </x:c>
+      <x:c r="D68" s="6" t="n">
+        <x:v>0.991748850166246</x:v>
+      </x:c>
+      <x:c r="E68" s="6" t="n">
+        <x:v>0.9739837398373984</x:v>
+      </x:c>
+      <x:c r="F68" s="6" t="n">
+        <x:v>0.9827766270407694</x:v>
+      </x:c>
+      <x:c r="G68" s="6" t="str">
+        <x:v>mean 3 seed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="24" customHeight="1">
+      <x:c r="A69" s="6" t="str">
+        <x:v>T00</x:v>
+      </x:c>
+      <x:c r="B69" s="6" t="str">
+        <x:v>Prickly acacia</x:v>
+      </x:c>
+      <x:c r="C69" s="9" t="n">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="D69" s="6" t="n">
+        <x:v>0.9254314802844216</x:v>
+      </x:c>
+      <x:c r="E69" s="6" t="n">
+        <x:v>0.970266040688576</x:v>
+      </x:c>
+      <x:c r="F69" s="6" t="n">
+        <x:v>0.9473047640523431</x:v>
+      </x:c>
+      <x:c r="G69" s="6" t="str">
+        <x:v>mean 3 seed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="24" customHeight="1">
+      <x:c r="A70" s="6" t="str">
+        <x:v>T00</x:v>
+      </x:c>
+      <x:c r="B70" s="6" t="str">
+        <x:v>Rubber vine</x:v>
+      </x:c>
+      <x:c r="C70" s="9" t="n">
+        <x:v>202</x:v>
+      </x:c>
+      <x:c r="D70" s="6" t="n">
+        <x:v>0.9819827210890629</x:v>
+      </x:c>
+      <x:c r="E70" s="6" t="n">
+        <x:v>0.9818481848184818</x:v>
+      </x:c>
+      <x:c r="F70" s="6" t="n">
+        <x:v>0.9818636075763655</x:v>
+      </x:c>
+      <x:c r="G70" s="6" t="str">
+        <x:v>mean 3 seed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="24" customHeight="1">
+      <x:c r="A71" s="6" t="str">
+        <x:v>T00</x:v>
+      </x:c>
+      <x:c r="B71" s="6" t="str">
+        <x:v>Siam weed</x:v>
+      </x:c>
+      <x:c r="C71" s="9" t="n">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="D71" s="6" t="n">
+        <x:v>0.9640464317528538</x:v>
+      </x:c>
+      <x:c r="E71" s="6" t="n">
+        <x:v>0.9937984496124032</x:v>
+      </x:c>
+      <x:c r="F71" s="6" t="n">
+        <x:v>0.978655341765673</x:v>
+      </x:c>
+      <x:c r="G71" s="6" t="str">
+        <x:v>mean 3 seed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="24" customHeight="1">
+      <x:c r="A72" s="6" t="str">
+        <x:v>T00</x:v>
+      </x:c>
+      <x:c r="B72" s="6" t="str">
+        <x:v>Snake weed</x:v>
+      </x:c>
+      <x:c r="C72" s="9" t="n">
+        <x:v>204</x:v>
+      </x:c>
+      <x:c r="D72" s="6" t="n">
+        <x:v>0.9462039003831705</x:v>
+      </x:c>
+      <x:c r="E72" s="6" t="n">
+        <x:v>0.9477124183006537</x:v>
+      </x:c>
+      <x:c r="F72" s="6" t="n">
+        <x:v>0.9468724678573968</x:v>
+      </x:c>
+      <x:c r="G72" s="6" t="str">
+        <x:v>mean 3 seed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="24" customHeight="1">
+      <x:c r="A73" s="6" t="str">
+        <x:v>T00</x:v>
+      </x:c>
+      <x:c r="B73" s="6" t="str">
+        <x:v>Negative</x:v>
+      </x:c>
+      <x:c r="C73" s="9" t="n">
+        <x:v>1822</x:v>
+      </x:c>
+      <x:c r="D73" s="6" t="n">
+        <x:v>0.9874817356750842</x:v>
+      </x:c>
+      <x:c r="E73" s="6" t="n">
+        <x:v>0.9811562385656787</x:v>
+      </x:c>
+      <x:c r="F73" s="6" t="n">
+        <x:v>0.9843063062050353</x:v>
+      </x:c>
+      <x:c r="G73" s="6" t="str">
+        <x:v>mean 3 seed</x:v>
+      </x:c>
     </x:row>
     <x:row r="74">
       <x:c r="C74" s="10"/>

</xml_diff>